<commit_message>
Complete GPT-6 Astra evidence record
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-four-year-capability-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-four-year-capability-report-card.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9a0940a3125d4bb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="2" r:id="R8da8e13224474d8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="3" r:id="R1ef87d98bcbd4838"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Path" sheetId="4" r:id="R697aab421d234433"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METR Horizon" sheetId="5" r:id="R5aab6667b7644f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Evidence" sheetId="6" r:id="R43b117debd5e4831"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Releases" sheetId="7" r:id="R75d07812935a4169"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rb8ccdc4d4c1d4fca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5e220b784f5f455a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="2" r:id="Rcc9bca2cbffc486c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="3" r:id="R3190523cbaeb436b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Path" sheetId="4" r:id="R27784fc422134033"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METR Horizon" sheetId="5" r:id="Rc0cd1f46f15f4780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Evidence" sheetId="6" r:id="Rce850d236b7e40c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Releases" sheetId="7" r:id="R6b2e9d8f177e4470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Re64be198ddcc4157"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -434,7 +434,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf692cba597744bfa"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcdcdc42325374d4a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -537,7 +537,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="CapabilityResearchEvidenceTable" displayName="CapabilityResearchEvidenceTable" ref="A5:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="CapabilityResearchEvidenceTable" displayName="CapabilityResearchEvidenceTable" ref="A5:I57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Category"/>
@@ -1207,7 +1207,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1109f040a14438b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09387638196847e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2538,7 +2538,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67a02012d48a4e8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc34ca3276aee40e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3919,7 +3919,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12261a76a63a4b8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R632a86f1ba8548cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4418,9 +4418,9 @@
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R965847d0cb314e76"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3d9885d5bf1475d"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b24a39c91640a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85c1e0ddf3454318"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4920,7 +4920,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34da4859e8644913"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd2377f340ec480c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6447,6 +6447,64 @@
         <x:v>Vendor-reported Elo. It remains ungraded because the forecast contract forbids rescaling a leaderboard without a fixed reference opponent or stable win-rate transformation.</x:v>
       </x:c>
     </x:row>
+    <x:row r="56" ht="183.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A56" s="16" t="str">
+        <x:v>evidence-051</x:v>
+      </x:c>
+      <x:c r="B56" s="16" t="str">
+        <x:v>Abstract reasoning</x:v>
+      </x:c>
+      <x:c r="C56" s="25" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="D56" s="16" t="str">
+        <x:v>GPT-6 Astra</x:v>
+      </x:c>
+      <x:c r="E56" s="16" t="str">
+        <x:v>FrontierMath Tier 4 score</x:v>
+      </x:c>
+      <x:c r="F56" s="16" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="G56" s="16" t="str">
+        <x:v>percent</x:v>
+      </x:c>
+      <x:c r="H56" s="16" t="str">
+        <x:v>gate1-openai-com-gpt-6-astra-release</x:v>
+      </x:c>
+      <x:c r="I56" s="16" t="str">
+        <x:v>Vendor-reported maximum-at-any-effort result on a frontier mathematical-reasoning benchmark. It is important capability evidence but not a direct economic-delegation outcome.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="172.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A57" s="16" t="str">
+        <x:v>evidence-052</x:v>
+      </x:c>
+      <x:c r="B57" s="16" t="str">
+        <x:v>Cybersecurity</x:v>
+      </x:c>
+      <x:c r="C57" s="25" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="D57" s="16" t="str">
+        <x:v>GPT-6 Astra</x:v>
+      </x:c>
+      <x:c r="E57" s="16" t="str">
+        <x:v>ExploitBench score</x:v>
+      </x:c>
+      <x:c r="F57" s="16" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G57" s="16" t="str">
+        <x:v>percent</x:v>
+      </x:c>
+      <x:c r="H57" s="16" t="str">
+        <x:v>gate1-openai-com-gpt-6-astra-release</x:v>
+      </x:c>
+      <x:c r="I57" s="16" t="str">
+        <x:v>Vendor-reported maximum-at-any-effort result. OpenAI designates Astra Critical capability in cyber; this is a capability and safety signal, not a Personal-AI delegation measure.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I2"/>
@@ -6454,7 +6512,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21276c5d015e4247"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9395d064228c4adf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7048,7 +7106,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc5f3d87c9c84734"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd768d4e6b564a47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8709,7 +8767,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5075f70358e9475c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36c1322c595e4f54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>